<commit_message>
feat(system): wire up missing tool pages - forms, automations, call analyzer, partners
- feat: add 'כלים' nav group with forms, automations, call analyzer, partners
- feat: create /forms route → FormsView (form builder with AI generation)
- feat: create /automations route → AutomationsView
- feat: create /call_analyzer route → CallAnalyzerView (sales call upload + AI)
- feat: create /partners route → PartnersView (affiliates tracking)
- feat: add loading skeletons for all new routes
- feat: register all new tabs in SHELL_TABS
- perf: memoize dashboard computed values (myLeads, hitListLeads, myTasks, nextMeeting)
</commit_message>
<xml_diff>
--- a/bot/misrad-ai-whatsapp-bot.xlsx
+++ b/bot/misrad-ai-whatsapp-bot.xlsx
@@ -571,7 +571,8 @@
 description:``
 (/item)
 &gt;
-(/list)</v>
+(/list)
+</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -701,7 +702,8 @@
 description:``
 (/item)
 &gt;
-(/list)</v>
+(/list)
+</v>
       </c>
       <c r="D3" t="str">
         <v/>
@@ -790,7 +792,7 @@
         <v/>
       </c>
       <c r="B4" t="str">
-        <v>------------------------------</v>
+        <v>----------------------------------------------------------</v>
       </c>
       <c r="C4" t="str">
         <v xml:space="preserve"> </v>
@@ -928,7 +930,8 @@
 description:``
 (/item)
 &gt;
-(/list)</v>
+(/list)
+</v>
       </c>
       <c r="D5" t="str">
         <v/>
@@ -1059,7 +1062,8 @@
 description:``
 (/item)
 &gt;
-(/list)</v>
+(/list)
+</v>
       </c>
       <c r="D6" t="str">
         <v/>
@@ -1798,7 +1802,8 @@
 description:``
 (/item)
 &gt;
-(/list)</v>
+(/list)
+</v>
       </c>
       <c r="D13" t="str">
         <v/>
@@ -1887,7 +1892,7 @@
         <v/>
       </c>
       <c r="B14" t="str">
-        <v>------------------------------</v>
+        <v>----------------------------------------------------------</v>
       </c>
       <c r="C14" t="str">
         <v xml:space="preserve"> </v>
@@ -2008,7 +2013,8 @@
 description:`ארגון גדול`
 (/item)
 &gt;
-(/list)</v>
+(/list)
+</v>
       </c>
       <c r="D15" t="str">
         <v/>
@@ -2126,7 +2132,8 @@
 description:``
 (/item)
 &gt;
-(/list)</v>
+(/list)
+</v>
       </c>
       <c r="D16" t="str">
         <v/>
@@ -2253,7 +2260,8 @@
 description:`נחבר אותך ליועץ`
 (/item)
 &gt;
-(/list)</v>
+(/list)
+</v>
       </c>
       <c r="D17" t="str">
         <v/>
@@ -2373,7 +2381,8 @@
 description:``
 (/item)
 &gt;
-(/list)</v>
+(/list)
+</v>
       </c>
       <c r="D18" t="str">
         <v/>
@@ -2493,7 +2502,8 @@
 description:``
 (/item)
 &gt;
-(/list)</v>
+(/list)
+</v>
       </c>
       <c r="D19" t="str">
         <v/>
@@ -2612,7 +2622,8 @@
 description:``
 (/item)
 &gt;
-(/list)</v>
+(/list)
+</v>
       </c>
       <c r="D20" t="str">
         <v/>
@@ -2735,7 +2746,8 @@
 description:``
 (/item)
 &gt;
-(/list)</v>
+(/list)
+</v>
       </c>
       <c r="D21" t="str">
         <v/>
@@ -2949,7 +2961,8 @@
 description:``
 (/item)
 &gt;
-(/list)</v>
+(/list)
+</v>
       </c>
       <c r="D23" t="str">
         <v/>
@@ -3038,7 +3051,7 @@
         <v/>
       </c>
       <c r="B24" t="str">
-        <v>------------------------------</v>
+        <v>----------------------------------------------------------</v>
       </c>
       <c r="C24" t="str">
         <v xml:space="preserve"> </v>
@@ -3246,7 +3259,8 @@
 description:``
 (/item)
 &gt;
-(/list)</v>
+(/list)
+</v>
       </c>
       <c r="D26" t="str">
         <v/>
@@ -3736,7 +3750,8 @@
 description:``
 (/item)
 &gt;
-(/list)</v>
+(/list)
+</v>
       </c>
       <c r="D31" t="str">
         <v/>
@@ -4020,7 +4035,7 @@
         <v/>
       </c>
       <c r="B34" t="str">
-        <v>------------------------------</v>
+        <v>----------------------------------------------------------</v>
       </c>
       <c r="C34" t="str">
         <v xml:space="preserve"> </v>
@@ -4329,7 +4344,8 @@
 description:``
 (/item)
 &gt;
-(/list)</v>
+(/list)
+</v>
       </c>
       <c r="D37" t="str">
         <v/>
@@ -4518,7 +4534,7 @@
         <v/>
       </c>
       <c r="B39" t="str">
-        <v>------------------------------</v>
+        <v>----------------------------------------------------------</v>
       </c>
       <c r="C39" t="str">
         <v xml:space="preserve"> </v>
@@ -4647,7 +4663,8 @@
 description:`מענה אנושי`
 (/item)
 &gt;
-(/list)</v>
+(/list)
+</v>
       </c>
       <c r="D40" t="str">
         <v/>
@@ -4768,7 +4785,8 @@
 description:``
 (/item)
 &gt;
-(/list)</v>
+(/list)
+</v>
       </c>
       <c r="D41" t="str">
         <v/>
@@ -5826,7 +5844,7 @@
         <v/>
       </c>
       <c r="B52" t="str">
-        <v>------------------------------</v>
+        <v>----------------------------------------------------------</v>
       </c>
       <c r="C52" t="str">
         <v xml:space="preserve"> </v>
@@ -6016,7 +6034,7 @@
         <v/>
       </c>
       <c r="B54" t="str">
-        <v>------------------------------</v>
+        <v>----------------------------------------------------------</v>
       </c>
       <c r="C54" t="str">
         <v xml:space="preserve"> </v>
@@ -6297,7 +6315,7 @@
         <v/>
       </c>
       <c r="B57" t="str">
-        <v>------------------------------</v>
+        <v>----------------------------------------------------------</v>
       </c>
       <c r="C57" t="str">
         <v xml:space="preserve"> </v>
@@ -6678,7 +6696,7 @@
         <v/>
       </c>
       <c r="B61" t="str">
-        <v>------------------------------</v>
+        <v>----------------------------------------------------------</v>
       </c>
       <c r="C61" t="str">
         <v xml:space="preserve"> </v>
@@ -6894,7 +6912,8 @@
 description:``
 (/item)
 &gt;
-(/list)</v>
+(/list)
+</v>
       </c>
       <c r="D63" t="str">
         <v/>
@@ -7178,7 +7197,7 @@
         <v/>
       </c>
       <c r="B66" t="str">
-        <v>------------------------------</v>
+        <v>----------------------------------------------------------</v>
       </c>
       <c r="C66" t="str">
         <v xml:space="preserve"> </v>

</xml_diff>